<commit_message>
Align data-entry templates with the live tool
Engagements template:
- Uniform red header row (was split red/navy by required vs optional)
- Engagement type dropdown trimmed from 6 to the 4 the tool actually
  offers (removed Email, Others), Instructions sheet and data
  validation range updated to match

Opportunities template:
- Uniform red header row, same as above
- Estimated value relabeled from USD to SGD
- Stage dropdown and Instructions text stripped of leading numbers
  ("01 Blue Sky Opportunity" -> "Blue Sky Opportunity"), matching the
  tool's LOOKUPS.opportunityStatus

Companies template intentionally left untouched - was never in scope.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Master/Engagements_Data_Entry_Template.xlsx
+++ b/Master/Engagements_Data_Entry_Template.xlsx
@@ -506,12 +506,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:A26"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
@@ -625,7 +626,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>• Engagement type *: In-Person Meeting, Virtual Meeting, Phone Call/ Whatsapp, Email, Conference/Event, Others</t>
+          <t>• Engagement type *: In-Person Meeting, Virtual Meeting, Phone Call/ Whatsapp, Conference/Event</t>
         </is>
       </c>
     </row>
@@ -724,7 +725,7 @@
           <t>BD / PM *</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Accompanied by</t>
         </is>
@@ -5911,7 +5912,7 @@
       <formula1>1900-01-01</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G302" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list">
-      <formula1>=Lists!$G$2:$G$7</formula1>
+      <formula1>=Lists!$G$2:$G$5</formula1>
     </dataValidation>
     <dataValidation sqref="H3:H302" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list">
       <formula1>=Lists!$H$2:$H$4</formula1>
@@ -6048,7 +6049,7 @@
     <row r="5">
       <c r="G5" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Conference/Event</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6063,11 +6064,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Conference/Event</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>Capability presentation</t>
@@ -6080,11 +6076,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Request for referral</t>

</xml_diff>